<commit_message>
Version 0.0.1 - Development
</commit_message>
<xml_diff>
--- a/Doc/程式歷程.xlsx
+++ b/Doc/程式歷程.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pgkamars\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\Side_Project\GifComposerWpf\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B728A533-10CF-40FB-9672-78D5E89CFDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4FF9C0-6CB6-4484-8272-915A0F42A74E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="開發階段" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="81">
   <si>
     <t>版本</t>
   </si>
@@ -232,6 +232,90 @@
   </si>
   <si>
     <t>名稱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FluentIcons.Wpf</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NuGet 套件</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ButtonStyles.xaml</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>iconBtnStyle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026.08.02</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Style</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>建立含有 icon 與文字的按鈕樣式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>iconTextBtnStyle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>建立只有 icon 按鈕樣式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TextBlockStyles.xaml</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>titleStyle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>hintTextStyle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>labelStyle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>標題文字樣式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>提示文字樣式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>標籤文字樣式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MainWindow.xaml</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>主畫面</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>新增圖片按鈕；刪除全部圖片按鈕；
+圖片列表；刪除圖片按鈕；上移按鈕；
+下移按鈕；拖曳圖片區塊；預覽圖片區塊；
+尺寸設定；循環次數設定；輸出路徑設定；
+產生 gif 按鈕；狀態列</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -658,7 +742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -753,6 +837,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1222,15 +1309,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5" style="5" customWidth="1"/>
     <col min="2" max="2" width="24.125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="16.25" style="5" customWidth="1"/>
+    <col min="3" max="3" width="30.375" style="5" customWidth="1"/>
     <col min="4" max="4" width="9" style="5"/>
     <col min="5" max="5" width="36.125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="51.625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="51.625" style="21" customWidth="1"/>
     <col min="7" max="7" width="32.625" style="5" customWidth="1"/>
     <col min="8" max="8" width="26" style="5" customWidth="1"/>
     <col min="9" max="16384" width="9" style="5"/>
@@ -1262,38 +1349,161 @@
         <v>24</v>
       </c>
     </row>
+    <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="B2:B80">
+  <conditionalFormatting sqref="B2:B208">
     <cfRule type="expression" dxfId="13" priority="1">
-      <formula>$B$2="Other"</formula>
+      <formula>B2="Other"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="12" priority="2">
-      <formula>$B$2="Resource"</formula>
+      <formula>B2="Resource"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="11" priority="4">
-      <formula>$B$2="Helper / Utility"</formula>
+      <formula>B2="Helper / Utility"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="10" priority="5">
-      <formula>$B$2="Converter"</formula>
+      <formula>B2="Converter"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="9" priority="6">
-      <formula>$B$2="Repository"</formula>
+      <formula>B2="Repository"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="8" priority="7">
-      <formula>$B$2="Service"</formula>
+      <formula>B2="Service"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="7" priority="8">
-      <formula>$B$2="Model"</formula>
+      <formula>B2="Model"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="6" priority="9">
-      <formula>$B$2="ViewModel"</formula>
+      <formula>B2="ViewModel"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="5" priority="10">
-      <formula>$B$2="View"</formula>
+      <formula>B2="View"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D80">
+  <conditionalFormatting sqref="D2:D208">
     <cfRule type="expression" dxfId="4" priority="11">
       <formula>D2="新增"</formula>
     </cfRule>
@@ -1319,13 +1529,13 @@
           <x14:formula1>
             <xm:f>選單!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D80</xm:sqref>
+          <xm:sqref>D2:D208</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F6C556B4-03A7-4A00-A5BF-2BB818AC178A}">
           <x14:formula1>
             <xm:f>選單!$D$2:$D$10</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B80</xm:sqref>
+          <xm:sqref>B2:B208</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1335,20 +1545,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B193875-8373-4603-8186-2E01BA7DA4CE}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="19.8" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9" style="5"/>
+    <col min="1" max="1" width="37.75" style="5" customWidth="1"/>
     <col min="2" max="2" width="23.375" style="5" customWidth="1"/>
     <col min="3" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="32" t="s">
         <v>60</v>
       </c>
       <c r="B1" s="32" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>